<commit_message>
Clean Moodle Publish workbook synchronization schema
</commit_message>
<xml_diff>
--- a/templates/AI_Curriculum_Workbook_v4.0_Production.xlsx
+++ b/templates/AI_Curriculum_Workbook_v4.0_Production.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11108"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/docker/curriculum-builder/templates/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5BB8664-29A9-514F-8FE5-DA2CB2AD006C}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E1B1ED0-CCDA-4852-B83B-95FA863D3435}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8380" yWindow="3660" windowWidth="28040" windowHeight="12720" firstSheet="3" activeTab="4" xr2:uid="{9649AE17-D6D9-6B47-A5D5-E2E16CE2B556}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="3" activeTab="16" xr2:uid="{9649AE17-D6D9-6B47-A5D5-E2E16CE2B556}"/>
   </bookViews>
   <sheets>
     <sheet name="Build_Metadata" sheetId="1" r:id="rId1"/>
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="542" uniqueCount="364">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="535" uniqueCount="359">
   <si>
     <t>build_id</t>
   </si>
@@ -135,9 +135,6 @@
     <t>section_id</t>
   </si>
   <si>
-    <t>page_id</t>
-  </si>
-  <si>
     <t>activity_url</t>
   </si>
   <si>
@@ -151,9 +148,6 @@
   </si>
   <si>
     <t>last_sync</t>
-  </si>
-  <si>
-    <t>cmid</t>
   </si>
   <si>
     <t>pptx</t>
@@ -1073,9 +1067,6 @@
     <t>recap_description</t>
   </si>
   <si>
-    <t>mission_pageid</t>
-  </si>
-  <si>
     <t>mission_cmid</t>
   </si>
   <si>
@@ -1085,13 +1076,7 @@
     <t>quiz_cmid</t>
   </si>
   <si>
-    <t>activities_pageid</t>
-  </si>
-  <si>
     <t>activities_cmid</t>
-  </si>
-  <si>
-    <t>recap_pageid</t>
   </si>
   <si>
     <t>recap_cmid</t>
@@ -1182,7 +1167,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="9">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1362,9 +1347,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1402,7 +1387,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1508,7 +1493,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1650,7 +1635,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1659,30 +1644,30 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{24285624-FCB6-3646-94CC-FE92EAF05548}">
   <dimension ref="A1:N1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75"/>
   <cols>
     <col min="1" max="1" width="7.5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.83203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.83203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="6.83203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6.875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="6" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="11" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.1640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="16.33203125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="16.375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.375" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="9.5" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="10.5" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="13" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:14">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C1" s="5" t="s">
         <v>1</v>
@@ -1718,7 +1703,7 @@
         <v>11</v>
       </c>
       <c r="N1" s="5" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
     </row>
   </sheetData>
@@ -1729,17 +1714,17 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7176D2CF-0D41-B348-B797-0B70B105DCFF}">
   <dimension ref="A1:J1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="20" style="7" customWidth="1"/>
     <col min="2" max="6" width="18" style="7" customWidth="1"/>
     <col min="7" max="7" width="19" style="7" customWidth="1"/>
     <col min="8" max="9" width="18" style="7" customWidth="1"/>
-    <col min="10" max="10" width="8.1640625" style="7" bestFit="1" customWidth="1"/>
-    <col min="11" max="16384" width="8.83203125" style="7"/>
+    <col min="10" max="10" width="8.125" style="7" bestFit="1" customWidth="1"/>
+    <col min="11" max="16384" width="8.875" style="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10">
       <c r="A1" s="6" t="s">
         <v>12</v>
       </c>
@@ -1747,28 +1732,28 @@
         <v>13</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="D1" s="6" t="s">
         <v>15</v>
       </c>
       <c r="E1" s="6" t="s">
+        <v>284</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>285</v>
+      </c>
+      <c r="G1" s="6" t="s">
+        <v>246</v>
+      </c>
+      <c r="H1" s="6" t="s">
         <v>286</v>
       </c>
-      <c r="F1" s="6" t="s">
-        <v>287</v>
-      </c>
-      <c r="G1" s="6" t="s">
-        <v>248</v>
-      </c>
-      <c r="H1" s="6" t="s">
-        <v>288</v>
-      </c>
       <c r="I1" s="6" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="J1" s="6" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -1780,88 +1765,88 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2103EC19-A556-664A-AE61-8EE4FB1F91E6}">
   <dimension ref="A1:P14"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="12" width="18" style="7" customWidth="1"/>
-    <col min="13" max="15" width="8.83203125" style="7"/>
+    <col min="13" max="15" width="8.875" style="7"/>
     <col min="16" max="16" width="12.5" style="7" bestFit="1" customWidth="1"/>
-    <col min="17" max="16384" width="8.83203125" style="7"/>
+    <col min="17" max="16384" width="8.875" style="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:16">
       <c r="A1" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>175</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>176</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>177</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="G1" s="6" t="s">
+        <v>180</v>
+      </c>
+      <c r="H1" s="6" t="s">
+        <v>181</v>
+      </c>
+      <c r="I1" s="6" t="s">
+        <v>182</v>
+      </c>
+      <c r="J1" s="6" t="s">
+        <v>183</v>
+      </c>
+      <c r="K1" s="6" t="s">
+        <v>184</v>
+      </c>
+      <c r="L1" s="6" t="s">
+        <v>185</v>
+      </c>
+      <c r="M1" s="6" t="s">
+        <v>186</v>
+      </c>
+      <c r="N1" s="6" t="s">
+        <v>187</v>
+      </c>
+      <c r="O1" s="6" t="s">
+        <v>188</v>
+      </c>
+      <c r="P1" s="6" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" ht="45">
+      <c r="A2" s="8" t="s">
+        <v>189</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>190</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>191</v>
+      </c>
+      <c r="D2" s="8" t="s">
+        <v>192</v>
+      </c>
+      <c r="E2" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="B1" s="6" t="s">
-        <v>177</v>
-      </c>
-      <c r="C1" s="6" t="s">
-        <v>178</v>
-      </c>
-      <c r="D1" s="6" t="s">
-        <v>179</v>
-      </c>
-      <c r="E1" s="6" t="s">
-        <v>180</v>
-      </c>
-      <c r="F1" s="6" t="s">
-        <v>181</v>
-      </c>
-      <c r="G1" s="6" t="s">
-        <v>182</v>
-      </c>
-      <c r="H1" s="6" t="s">
-        <v>183</v>
-      </c>
-      <c r="I1" s="6" t="s">
-        <v>184</v>
-      </c>
-      <c r="J1" s="6" t="s">
-        <v>185</v>
-      </c>
-      <c r="K1" s="6" t="s">
-        <v>186</v>
-      </c>
-      <c r="L1" s="6" t="s">
-        <v>187</v>
-      </c>
-      <c r="M1" s="6" t="s">
-        <v>188</v>
-      </c>
-      <c r="N1" s="6" t="s">
-        <v>189</v>
-      </c>
-      <c r="O1" s="6" t="s">
-        <v>190</v>
-      </c>
-      <c r="P1" s="6" t="s">
-        <v>297</v>
-      </c>
-    </row>
-    <row r="2" spans="1:16" ht="48" x14ac:dyDescent="0.2">
-      <c r="A2" s="8" t="s">
-        <v>191</v>
-      </c>
-      <c r="B2" s="8" t="s">
-        <v>192</v>
-      </c>
-      <c r="C2" s="8" t="s">
+      <c r="F2" s="8" t="s">
         <v>193</v>
       </c>
-      <c r="D2" s="8" t="s">
+      <c r="G2" s="8" t="s">
         <v>194</v>
       </c>
-      <c r="E2" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="F2" s="8" t="s">
+      <c r="H2" s="8" t="s">
         <v>195</v>
-      </c>
-      <c r="G2" s="8" t="s">
-        <v>196</v>
-      </c>
-      <c r="H2" s="8" t="s">
-        <v>197</v>
       </c>
       <c r="I2" s="8">
         <v>0.3</v>
@@ -1870,7 +1855,7 @@
         <v>2000</v>
       </c>
       <c r="K2" s="8" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="L2" s="8"/>
       <c r="M2" s="8" t="b">
@@ -1880,33 +1865,33 @@
         <v>1</v>
       </c>
       <c r="O2" s="8" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" ht="30">
+      <c r="A3" s="8" t="s">
+        <v>198</v>
+      </c>
+      <c r="B3" s="8" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="3" spans="1:16" ht="32" x14ac:dyDescent="0.2">
-      <c r="A3" s="8" t="s">
+      <c r="C3" s="8" t="s">
         <v>200</v>
       </c>
-      <c r="B3" s="8" t="s">
-        <v>201</v>
-      </c>
-      <c r="C3" s="8" t="s">
-        <v>202</v>
-      </c>
       <c r="D3" s="8" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F3" s="8" t="s">
+        <v>193</v>
+      </c>
+      <c r="G3" s="8" t="s">
+        <v>194</v>
+      </c>
+      <c r="H3" s="8" t="s">
         <v>195</v>
-      </c>
-      <c r="G3" s="8" t="s">
-        <v>196</v>
-      </c>
-      <c r="H3" s="8" t="s">
-        <v>197</v>
       </c>
       <c r="I3" s="8">
         <v>0.4</v>
@@ -1915,10 +1900,10 @@
         <v>2500</v>
       </c>
       <c r="K3" s="8" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="L3" s="8" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="M3" s="8" t="b">
         <v>1</v>
@@ -1927,33 +1912,33 @@
         <v>1</v>
       </c>
       <c r="O3" s="8" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" ht="45">
+      <c r="A4" s="8" t="s">
+        <v>203</v>
+      </c>
+      <c r="B4" s="8" t="s">
         <v>204</v>
       </c>
-    </row>
-    <row r="4" spans="1:16" ht="48" x14ac:dyDescent="0.2">
-      <c r="A4" s="8" t="s">
-        <v>205</v>
-      </c>
-      <c r="B4" s="8" t="s">
-        <v>206</v>
-      </c>
       <c r="C4" s="8" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="D4" s="8" t="s">
         <v>20</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="H4" s="8" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="I4" s="8">
         <v>0.5</v>
@@ -1962,10 +1947,10 @@
         <v>8000</v>
       </c>
       <c r="K4" s="8" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="L4" s="8" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="M4" s="8" t="b">
         <v>1</v>
@@ -1974,33 +1959,33 @@
         <v>1</v>
       </c>
       <c r="O4" s="8" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" ht="30">
+      <c r="A5" s="8" t="s">
+        <v>208</v>
+      </c>
+      <c r="B5" s="8" t="s">
         <v>209</v>
       </c>
-    </row>
-    <row r="5" spans="1:16" ht="32" x14ac:dyDescent="0.2">
-      <c r="A5" s="8" t="s">
-        <v>210</v>
-      </c>
-      <c r="B5" s="8" t="s">
-        <v>211</v>
-      </c>
       <c r="C5" s="8" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F5" s="8" t="s">
+        <v>193</v>
+      </c>
+      <c r="G5" s="8" t="s">
+        <v>194</v>
+      </c>
+      <c r="H5" s="8" t="s">
         <v>195</v>
-      </c>
-      <c r="G5" s="8" t="s">
-        <v>196</v>
-      </c>
-      <c r="H5" s="8" t="s">
-        <v>197</v>
       </c>
       <c r="I5" s="8">
         <v>0.4</v>
@@ -2009,10 +1994,10 @@
         <v>3000</v>
       </c>
       <c r="K5" s="8" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="L5" s="8" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="M5" s="8" t="b">
         <v>1</v>
@@ -2021,33 +2006,33 @@
         <v>1</v>
       </c>
       <c r="O5" s="8" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" ht="30">
+      <c r="A6" s="8" t="s">
+        <v>212</v>
+      </c>
+      <c r="B6" s="8" t="s">
         <v>213</v>
       </c>
-    </row>
-    <row r="6" spans="1:16" ht="32" x14ac:dyDescent="0.2">
-      <c r="A6" s="8" t="s">
-        <v>214</v>
-      </c>
-      <c r="B6" s="8" t="s">
-        <v>215</v>
-      </c>
       <c r="C6" s="8" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="D6" s="8" t="s">
         <v>19</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F6" s="8" t="s">
+        <v>193</v>
+      </c>
+      <c r="G6" s="8" t="s">
+        <v>194</v>
+      </c>
+      <c r="H6" s="8" t="s">
         <v>195</v>
-      </c>
-      <c r="G6" s="8" t="s">
-        <v>196</v>
-      </c>
-      <c r="H6" s="8" t="s">
-        <v>197</v>
       </c>
       <c r="I6" s="8">
         <v>0.3</v>
@@ -2056,10 +2041,10 @@
         <v>1500</v>
       </c>
       <c r="K6" s="8" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="L6" s="8" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="M6" s="8" t="b">
         <v>1</v>
@@ -2068,33 +2053,33 @@
         <v>1</v>
       </c>
       <c r="O6" s="8" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" ht="30">
+      <c r="A7" s="8" t="s">
+        <v>216</v>
+      </c>
+      <c r="B7" s="8" t="s">
         <v>217</v>
       </c>
-    </row>
-    <row r="7" spans="1:16" ht="32" x14ac:dyDescent="0.2">
-      <c r="A7" s="8" t="s">
-        <v>218</v>
-      </c>
-      <c r="B7" s="8" t="s">
-        <v>219</v>
-      </c>
       <c r="C7" s="8" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F7" s="8" t="s">
+        <v>193</v>
+      </c>
+      <c r="G7" s="8" t="s">
+        <v>194</v>
+      </c>
+      <c r="H7" s="8" t="s">
         <v>195</v>
-      </c>
-      <c r="G7" s="8" t="s">
-        <v>196</v>
-      </c>
-      <c r="H7" s="8" t="s">
-        <v>197</v>
       </c>
       <c r="I7" s="8">
         <v>0.2</v>
@@ -2103,10 +2088,10 @@
         <v>1500</v>
       </c>
       <c r="K7" s="8" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="L7" s="8" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="M7" s="8" t="b">
         <v>1</v>
@@ -2115,43 +2100,43 @@
         <v>1</v>
       </c>
       <c r="O7" s="8" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" ht="45">
+      <c r="A8" s="8" t="s">
+        <v>220</v>
+      </c>
+      <c r="B8" s="8" t="s">
         <v>221</v>
       </c>
-    </row>
-    <row r="8" spans="1:16" ht="48" x14ac:dyDescent="0.2">
-      <c r="A8" s="8" t="s">
+      <c r="C8" s="8" t="s">
         <v>222</v>
       </c>
-      <c r="B8" s="8" t="s">
+      <c r="D8" s="8" t="s">
+        <v>154</v>
+      </c>
+      <c r="E8" s="8" t="s">
         <v>223</v>
       </c>
-      <c r="C8" s="8" t="s">
+      <c r="F8" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="G8" s="8" t="s">
         <v>224</v>
       </c>
-      <c r="D8" s="8" t="s">
-        <v>156</v>
-      </c>
-      <c r="E8" s="8" t="s">
+      <c r="H8" s="8" t="s">
         <v>225</v>
-      </c>
-      <c r="F8" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="G8" s="8" t="s">
-        <v>226</v>
-      </c>
-      <c r="H8" s="8" t="s">
-        <v>227</v>
       </c>
       <c r="I8" s="8">
         <v>0</v>
       </c>
       <c r="J8" s="8"/>
       <c r="K8" s="8" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="L8" s="8" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="M8" s="8" t="b">
         <v>1</v>
@@ -2160,43 +2145,43 @@
         <v>1</v>
       </c>
       <c r="O8" s="8" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" ht="45">
+      <c r="A9" s="8" t="s">
+        <v>228</v>
+      </c>
+      <c r="B9" s="8" t="s">
         <v>229</v>
       </c>
-    </row>
-    <row r="9" spans="1:16" ht="48" x14ac:dyDescent="0.2">
-      <c r="A9" s="8" t="s">
+      <c r="C9" s="8" t="s">
+        <v>222</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>155</v>
+      </c>
+      <c r="E9" s="8" t="s">
         <v>230</v>
       </c>
-      <c r="B9" s="8" t="s">
+      <c r="F9" s="8" t="s">
         <v>231</v>
       </c>
-      <c r="C9" s="8" t="s">
-        <v>224</v>
-      </c>
-      <c r="D9" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="E9" s="8" t="s">
+      <c r="G9" s="8" t="s">
         <v>232</v>
       </c>
-      <c r="F9" s="8" t="s">
+      <c r="H9" s="8" t="s">
         <v>233</v>
-      </c>
-      <c r="G9" s="8" t="s">
-        <v>234</v>
-      </c>
-      <c r="H9" s="8" t="s">
-        <v>235</v>
       </c>
       <c r="I9" s="8">
         <v>0</v>
       </c>
       <c r="J9" s="8"/>
       <c r="K9" s="8" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="L9" s="8" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="M9" s="8" t="b">
         <v>1</v>
@@ -2205,33 +2190,33 @@
         <v>1</v>
       </c>
       <c r="O9" s="8" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" ht="45">
+      <c r="A10" s="8" t="s">
+        <v>236</v>
+      </c>
+      <c r="B10" s="8" t="s">
         <v>237</v>
       </c>
-    </row>
-    <row r="10" spans="1:16" ht="48" x14ac:dyDescent="0.2">
-      <c r="A10" s="8" t="s">
+      <c r="C10" s="8" t="s">
         <v>238</v>
       </c>
-      <c r="B10" s="8" t="s">
+      <c r="D10" s="8" t="s">
         <v>239</v>
       </c>
-      <c r="C10" s="8" t="s">
+      <c r="E10" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="F10" s="8" t="s">
         <v>240</v>
       </c>
-      <c r="D10" s="8" t="s">
-        <v>241</v>
-      </c>
-      <c r="E10" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="F10" s="8" t="s">
-        <v>242</v>
-      </c>
       <c r="G10" s="8" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="H10" s="8" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="I10" s="8">
         <v>0.3</v>
@@ -2240,10 +2225,10 @@
         <v>6000</v>
       </c>
       <c r="K10" s="8" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="L10" s="8" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="M10" s="8" t="b">
         <v>1</v>
@@ -2252,33 +2237,33 @@
         <v>1</v>
       </c>
       <c r="O10" s="8" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" ht="45">
+      <c r="A11" s="8" t="s">
+        <v>243</v>
+      </c>
+      <c r="B11" s="8" t="s">
         <v>244</v>
       </c>
-    </row>
-    <row r="11" spans="1:16" ht="48" x14ac:dyDescent="0.2">
-      <c r="A11" s="8" t="s">
+      <c r="C11" s="8" t="s">
         <v>245</v>
       </c>
-      <c r="B11" s="8" t="s">
+      <c r="D11" s="8" t="s">
         <v>246</v>
       </c>
-      <c r="C11" s="8" t="s">
-        <v>247</v>
-      </c>
-      <c r="D11" s="8" t="s">
-        <v>248</v>
-      </c>
       <c r="E11" s="8" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="H11" s="8" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="I11" s="8">
         <v>0.4</v>
@@ -2287,10 +2272,10 @@
         <v>5000</v>
       </c>
       <c r="K11" s="8" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="L11" s="8" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="M11" s="8" t="b">
         <v>1</v>
@@ -2299,33 +2284,33 @@
         <v>1</v>
       </c>
       <c r="O11" s="8" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" ht="30">
+      <c r="A12" s="8" t="s">
+        <v>249</v>
+      </c>
+      <c r="B12" s="8" t="s">
         <v>250</v>
       </c>
-    </row>
-    <row r="12" spans="1:16" ht="32" x14ac:dyDescent="0.2">
-      <c r="A12" s="8" t="s">
-        <v>251</v>
-      </c>
-      <c r="B12" s="8" t="s">
-        <v>252</v>
-      </c>
       <c r="C12" s="8" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="G12" s="8" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="H12" s="8" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="I12" s="8">
         <v>0.4</v>
@@ -2334,10 +2319,10 @@
         <v>5000</v>
       </c>
       <c r="K12" s="8" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="L12" s="8" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="M12" s="8" t="b">
         <v>1</v>
@@ -2346,43 +2331,43 @@
         <v>1</v>
       </c>
       <c r="O12" s="8" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="13" spans="1:16" ht="48" x14ac:dyDescent="0.2">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" ht="45">
       <c r="A13" s="8" t="s">
+        <v>252</v>
+      </c>
+      <c r="B13" s="8" t="s">
+        <v>253</v>
+      </c>
+      <c r="C13" s="8" t="s">
+        <v>245</v>
+      </c>
+      <c r="D13" s="8" t="s">
+        <v>246</v>
+      </c>
+      <c r="E13" s="8" t="s">
         <v>254</v>
       </c>
-      <c r="B13" s="8" t="s">
+      <c r="F13" s="8" t="s">
         <v>255</v>
       </c>
-      <c r="C13" s="8" t="s">
-        <v>247</v>
-      </c>
-      <c r="D13" s="8" t="s">
-        <v>248</v>
-      </c>
-      <c r="E13" s="8" t="s">
+      <c r="G13" s="8" t="s">
         <v>256</v>
       </c>
-      <c r="F13" s="8" t="s">
-        <v>257</v>
-      </c>
-      <c r="G13" s="8" t="s">
-        <v>258</v>
-      </c>
       <c r="H13" s="8" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="I13" s="8">
         <v>0</v>
       </c>
       <c r="J13" s="8"/>
       <c r="K13" s="8" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="L13" s="8" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="M13" s="8" t="b">
         <v>1</v>
@@ -2391,43 +2376,43 @@
         <v>1</v>
       </c>
       <c r="O13" s="8" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" ht="30">
+      <c r="A14" s="8" t="s">
+        <v>259</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>139</v>
+      </c>
+      <c r="C14" s="8" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="14" spans="1:16" ht="32" x14ac:dyDescent="0.2">
-      <c r="A14" s="8" t="s">
+      <c r="D14" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="E14" s="8" t="s">
         <v>261</v>
       </c>
-      <c r="B14" s="8" t="s">
-        <v>141</v>
-      </c>
-      <c r="C14" s="8" t="s">
+      <c r="F14" s="8" t="s">
         <v>262</v>
       </c>
-      <c r="D14" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="E14" s="8" t="s">
+      <c r="G14" s="8" t="s">
         <v>263</v>
       </c>
-      <c r="F14" s="8" t="s">
+      <c r="H14" s="8" t="s">
         <v>264</v>
-      </c>
-      <c r="G14" s="8" t="s">
-        <v>265</v>
-      </c>
-      <c r="H14" s="8" t="s">
-        <v>266</v>
       </c>
       <c r="I14" s="8">
         <v>0</v>
       </c>
       <c r="J14" s="8"/>
       <c r="K14" s="8" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="L14" s="8" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="M14" s="8" t="b">
         <v>1</v>
@@ -2436,7 +2421,7 @@
         <v>1</v>
       </c>
       <c r="O14" s="8" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
     </row>
   </sheetData>
@@ -2448,16 +2433,16 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD64F75D-F004-2440-AC25-6D9FC84CD08D}">
   <dimension ref="A1:L1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75"/>
   <cols>
-    <col min="1" max="1" width="15.1640625" customWidth="1"/>
-    <col min="3" max="3" width="14.83203125" customWidth="1"/>
-    <col min="8" max="8" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="5.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.125" customWidth="1"/>
+    <col min="3" max="3" width="14.875" customWidth="1"/>
+    <col min="8" max="8" width="9.625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="5.625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:12">
       <c r="A1" s="6" t="s">
         <v>12</v>
       </c>
@@ -2480,19 +2465,19 @@
         <v>6</v>
       </c>
       <c r="H1" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="I1" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="J1" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="K1" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="L1" s="5" t="s">
         <v>35</v>
-      </c>
-      <c r="K1" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="L1" s="5" t="s">
-        <v>37</v>
       </c>
     </row>
   </sheetData>
@@ -2503,7 +2488,7 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B97C3C44-A62B-2B40-A142-ADE1D0CC8BA9}">
   <dimension ref="A1:P1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="4" width="18" style="7" customWidth="1"/>
     <col min="5" max="5" width="19" style="7" customWidth="1"/>
@@ -2511,57 +2496,57 @@
     <col min="8" max="8" width="20" style="7" customWidth="1"/>
     <col min="9" max="15" width="18" style="7" customWidth="1"/>
     <col min="16" max="16" width="8" style="7" bestFit="1" customWidth="1"/>
-    <col min="17" max="16384" width="8.83203125" style="7"/>
+    <col min="17" max="16384" width="8.875" style="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:16">
       <c r="A1" s="6" t="s">
         <v>13</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="C1" s="6" t="s">
+        <v>267</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>149</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>268</v>
+      </c>
+      <c r="F1" s="6" t="s">
         <v>269</v>
       </c>
-      <c r="D1" s="6" t="s">
-        <v>151</v>
-      </c>
-      <c r="E1" s="6" t="s">
+      <c r="G1" s="6" t="s">
         <v>270</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="H1" s="6" t="s">
         <v>271</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="I1" s="6" t="s">
         <v>272</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="J1" s="6" t="s">
         <v>273</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="K1" s="6" t="s">
         <v>274</v>
       </c>
-      <c r="J1" s="6" t="s">
+      <c r="L1" s="6" t="s">
+        <v>182</v>
+      </c>
+      <c r="M1" s="6" t="s">
         <v>275</v>
       </c>
-      <c r="K1" s="6" t="s">
+      <c r="N1" s="6" t="s">
         <v>276</v>
       </c>
-      <c r="L1" s="6" t="s">
-        <v>184</v>
-      </c>
-      <c r="M1" s="6" t="s">
+      <c r="O1" s="6" t="s">
         <v>277</v>
       </c>
-      <c r="N1" s="6" t="s">
+      <c r="P1" s="6" t="s">
         <v>278</v>
-      </c>
-      <c r="O1" s="6" t="s">
-        <v>279</v>
-      </c>
-      <c r="P1" s="6" t="s">
-        <v>280</v>
       </c>
     </row>
   </sheetData>
@@ -2573,19 +2558,19 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77C51983-A67E-B549-977A-08CC4624482D}">
   <dimension ref="A1:Y1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75"/>
   <cols>
     <col min="8" max="8" width="13" customWidth="1"/>
-    <col min="9" max="9" width="13.6640625" customWidth="1"/>
-    <col min="10" max="10" width="15.83203125" customWidth="1"/>
-    <col min="18" max="18" width="13.83203125" customWidth="1"/>
-    <col min="19" max="19" width="13.6640625" customWidth="1"/>
-    <col min="20" max="20" width="12.33203125" customWidth="1"/>
-    <col min="21" max="21" width="12.1640625" customWidth="1"/>
+    <col min="9" max="9" width="13.625" customWidth="1"/>
+    <col min="10" max="10" width="15.875" customWidth="1"/>
+    <col min="18" max="18" width="13.875" customWidth="1"/>
+    <col min="19" max="19" width="13.625" customWidth="1"/>
+    <col min="20" max="20" width="12.375" customWidth="1"/>
+    <col min="21" max="21" width="12.125" customWidth="1"/>
     <col min="25" max="25" width="17.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:25">
       <c r="A1" s="5" t="s">
         <v>12</v>
       </c>
@@ -2593,73 +2578,73 @@
         <v>13</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="D1" s="5" t="s">
+        <v>151</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="F1" s="5" t="s">
         <v>153</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="G1" s="5" t="s">
         <v>154</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>155</v>
-      </c>
-      <c r="G1" s="5" t="s">
-        <v>156</v>
       </c>
       <c r="H1" s="5" t="s">
         <v>21</v>
       </c>
       <c r="I1" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="J1" s="5" t="s">
+        <v>156</v>
+      </c>
+      <c r="K1" s="5" t="s">
         <v>157</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="L1" s="5" t="s">
+        <v>172</v>
+      </c>
+      <c r="M1" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="N1" s="5" t="s">
         <v>158</v>
       </c>
-      <c r="K1" s="5" t="s">
+      <c r="O1" s="5" t="s">
         <v>159</v>
       </c>
-      <c r="L1" s="5" t="s">
-        <v>174</v>
-      </c>
-      <c r="M1" s="5" t="s">
-        <v>175</v>
-      </c>
-      <c r="N1" s="5" t="s">
+      <c r="P1" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="O1" s="5" t="s">
+      <c r="Q1" s="5" t="s">
         <v>161</v>
       </c>
-      <c r="P1" s="5" t="s">
+      <c r="R1" s="5" t="s">
         <v>162</v>
       </c>
-      <c r="Q1" s="5" t="s">
+      <c r="S1" s="5" t="s">
         <v>163</v>
       </c>
-      <c r="R1" s="5" t="s">
+      <c r="T1" s="5" t="s">
         <v>164</v>
       </c>
-      <c r="S1" s="5" t="s">
+      <c r="U1" s="5" t="s">
         <v>165</v>
       </c>
-      <c r="T1" s="5" t="s">
+      <c r="V1" s="5" t="s">
         <v>166</v>
       </c>
-      <c r="U1" s="5" t="s">
+      <c r="W1" s="5" t="s">
         <v>167</v>
       </c>
-      <c r="V1" s="5" t="s">
+      <c r="X1" s="5" t="s">
         <v>168</v>
       </c>
-      <c r="W1" s="5" t="s">
+      <c r="Y1" s="5" t="s">
         <v>169</v>
-      </c>
-      <c r="X1" s="5" t="s">
-        <v>170</v>
-      </c>
-      <c r="Y1" s="5" t="s">
-        <v>171</v>
       </c>
     </row>
   </sheetData>
@@ -2670,19 +2655,19 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D763B5A6-ADBF-C443-B73E-CFEDE782190B}">
   <dimension ref="A1:M1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75"/>
   <cols>
-    <col min="1" max="1" width="16.33203125" customWidth="1"/>
+    <col min="1" max="1" width="16.375" customWidth="1"/>
     <col min="2" max="2" width="12.5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.6640625" customWidth="1"/>
-    <col min="5" max="5" width="7.33203125" customWidth="1"/>
-    <col min="8" max="8" width="12.6640625" customWidth="1"/>
-    <col min="10" max="10" width="15.33203125" customWidth="1"/>
-    <col min="11" max="11" width="16.6640625" customWidth="1"/>
-    <col min="12" max="12" width="5.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.625" customWidth="1"/>
+    <col min="5" max="5" width="7.375" customWidth="1"/>
+    <col min="8" max="8" width="12.625" customWidth="1"/>
+    <col min="10" max="10" width="15.375" customWidth="1"/>
+    <col min="11" max="11" width="16.625" customWidth="1"/>
+    <col min="12" max="12" width="5.625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:13">
       <c r="A1" s="5" t="s">
         <v>12</v>
       </c>
@@ -2702,22 +2687,22 @@
         <v>6</v>
       </c>
       <c r="G1" s="5" t="s">
+        <v>305</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>306</v>
+      </c>
+      <c r="I1" s="5" t="s">
         <v>307</v>
       </c>
-      <c r="H1" s="5" t="s">
-        <v>308</v>
-      </c>
-      <c r="I1" s="5" t="s">
-        <v>309</v>
-      </c>
       <c r="J1" s="5" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="K1" s="6" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="L1" s="5" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="M1" s="5" t="s">
         <v>10</v>
@@ -2731,44 +2716,44 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{90331A06-603F-4C40-9F40-0A406A539AD2}">
   <dimension ref="A1:L1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75"/>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:12">
       <c r="A1" s="5" t="s">
         <v>12</v>
       </c>
       <c r="B1" s="5" t="s">
+        <v>342</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>343</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>344</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>345</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>346</v>
+      </c>
+      <c r="G1" s="5" t="s">
         <v>347</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="H1" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="I1" s="5" t="s">
         <v>348</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="J1" s="5" t="s">
         <v>349</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="K1" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="L1" s="5" t="s">
         <v>350</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>351</v>
-      </c>
-      <c r="G1" s="5" t="s">
-        <v>352</v>
-      </c>
-      <c r="H1" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="I1" s="5" t="s">
-        <v>353</v>
-      </c>
-      <c r="J1" s="5" t="s">
-        <v>354</v>
-      </c>
-      <c r="K1" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="L1" s="5" t="s">
-        <v>355</v>
       </c>
     </row>
   </sheetData>
@@ -2779,28 +2764,24 @@
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61F59446-E505-314D-AAA1-9A243212F6D6}">
-  <dimension ref="A1:AG1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:Z1"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75"/>
   <cols>
-    <col min="1" max="1" width="16.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12.5" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="7.6640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="7.625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14.625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.625" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="9" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="9.5" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="7.6640625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="5.1640625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="10.1640625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="16.33203125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="13.83203125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="8" bestFit="1" customWidth="1"/>
-    <col min="31" max="32" width="15.6640625" customWidth="1"/>
+    <col min="15" max="15" width="13.875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="12.375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="8" bestFit="1" customWidth="1"/>
+    <col min="24" max="25" width="15.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:33" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:26">
       <c r="A1" s="5" t="s">
         <v>12</v>
       </c>
@@ -2820,13 +2801,13 @@
         <v>5</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="H1" s="5" t="s">
         <v>6</v>
       </c>
       <c r="I1" s="5" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="J1" s="5" t="s">
         <v>13</v>
@@ -2844,61 +2825,40 @@
         <v>23</v>
       </c>
       <c r="O1" s="5" t="s">
-        <v>24</v>
+        <v>327</v>
       </c>
       <c r="P1" s="5" t="s">
-        <v>30</v>
+        <v>328</v>
       </c>
       <c r="Q1" s="5" t="s">
+        <v>329</v>
+      </c>
+      <c r="R1" s="5" t="s">
+        <v>330</v>
+      </c>
+      <c r="S1" s="5" t="s">
+        <v>331</v>
+      </c>
+      <c r="T1" s="5" t="s">
+        <v>332</v>
+      </c>
+      <c r="U1" s="5" t="s">
+        <v>333</v>
+      </c>
+      <c r="V1" s="5" t="s">
+        <v>334</v>
+      </c>
+      <c r="W1" s="5" t="s">
+        <v>335</v>
+      </c>
+      <c r="X1" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="Y1" s="5" t="s">
         <v>25</v>
-      </c>
-      <c r="R1" s="5" t="s">
-        <v>329</v>
-      </c>
-      <c r="S1" s="5" t="s">
-        <v>330</v>
-      </c>
-      <c r="T1" s="5" t="s">
-        <v>331</v>
-      </c>
-      <c r="U1" s="5" t="s">
-        <v>332</v>
-      </c>
-      <c r="V1" s="5" t="s">
-        <v>333</v>
-      </c>
-      <c r="W1" s="5" t="s">
-        <v>334</v>
-      </c>
-      <c r="X1" s="5" t="s">
-        <v>335</v>
-      </c>
-      <c r="Y1" s="5" t="s">
-        <v>336</v>
       </c>
       <c r="Z1" s="5" t="s">
         <v>27</v>
-      </c>
-      <c r="AA1" s="5" t="s">
-        <v>337</v>
-      </c>
-      <c r="AB1" s="5" t="s">
-        <v>338</v>
-      </c>
-      <c r="AC1" s="5" t="s">
-        <v>339</v>
-      </c>
-      <c r="AD1" s="5" t="s">
-        <v>340</v>
-      </c>
-      <c r="AE1" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="AF1" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="AG1" s="5" t="s">
-        <v>28</v>
       </c>
     </row>
   </sheetData>
@@ -2909,23 +2869,23 @@
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3DB8EA45-1F54-D040-A118-FACBB72EBE88}">
   <dimension ref="A1:E1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5">
       <c r="A1" s="5" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B1" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>38</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>40</v>
       </c>
     </row>
   </sheetData>
@@ -2936,601 +2896,601 @@
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B5AC78D4-4294-5844-922B-E81962E591A3}">
   <dimension ref="A1:A206"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75"/>
   <sheetData>
-    <row r="1" spans="1:1" ht="31" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:1" ht="31.5">
       <c r="A1" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" ht="23.25">
+      <c r="A3" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" ht="31.5">
+      <c r="A7" s="1" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="3" spans="1:1" ht="24" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
+    <row r="9" spans="1:1">
+      <c r="A9" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="7" spans="1:1" ht="31" x14ac:dyDescent="0.35">
-      <c r="A7" s="1" t="s">
+    <row r="11" spans="1:1">
+      <c r="A11" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
+    <row r="13" spans="1:1">
+      <c r="A13" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
+    <row r="17" spans="1:1" ht="31.5">
+      <c r="A17" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
+    <row r="19" spans="1:1">
+      <c r="A19" s="3" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="17" spans="1:1" ht="31" x14ac:dyDescent="0.35">
-      <c r="A17" s="1" t="s">
+    <row r="20" spans="1:1">
+      <c r="A20" s="3" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="19" spans="1:1" ht="17" x14ac:dyDescent="0.25">
-      <c r="A19" s="3" t="s">
+    <row r="21" spans="1:1">
+      <c r="A21" s="3" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="20" spans="1:1" ht="17" x14ac:dyDescent="0.25">
-      <c r="A20" s="3" t="s">
+    <row r="22" spans="1:1">
+      <c r="A22" s="3" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="21" spans="1:1" ht="17" x14ac:dyDescent="0.25">
-      <c r="A21" s="3" t="s">
+    <row r="23" spans="1:1">
+      <c r="A23" s="3" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1">
+      <c r="A24" s="3" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1">
+      <c r="A25" s="3" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="22" spans="1:1" ht="17" x14ac:dyDescent="0.25">
-      <c r="A22" s="3" t="s">
+    <row r="26" spans="1:1">
+      <c r="A26" s="3" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1">
+      <c r="A27" s="3" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1">
+      <c r="A28" s="3" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="23" spans="1:1" ht="17" x14ac:dyDescent="0.25">
-      <c r="A23" s="3" t="s">
+    <row r="29" spans="1:1">
+      <c r="A29" s="3" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1">
+      <c r="A30" s="3" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1">
+      <c r="A31" s="3" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1">
+      <c r="A32" s="3" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1">
+      <c r="A33" s="3" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1">
+      <c r="A34" s="3" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" ht="31.5">
+      <c r="A38" s="1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" ht="23.25">
+      <c r="A40" s="2" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1">
+      <c r="A42" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1">
+      <c r="A44" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1">
+      <c r="A46" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1">
+      <c r="A47" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="48" spans="1:1">
+      <c r="A48" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1">
+      <c r="A49" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1">
+      <c r="A50" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="51" spans="1:1">
+      <c r="A51" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="52" spans="1:1">
+      <c r="A52" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="53" spans="1:1">
+      <c r="A53" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="54" spans="1:1">
+      <c r="A54" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="55" spans="1:1">
+      <c r="A55" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="56" spans="1:1">
+      <c r="A56" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="57" spans="1:1">
+      <c r="A57" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="58" spans="1:1">
+      <c r="A58" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="60" spans="1:1">
+      <c r="A60" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="62" spans="1:1">
+      <c r="A62" s="4" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="66" spans="1:1" ht="23.25">
+      <c r="A66" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="68" spans="1:1">
+      <c r="A68" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="70" spans="1:1">
+      <c r="A70" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="72" spans="1:1">
+      <c r="A72" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="74" spans="1:1">
+      <c r="A74" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="75" spans="1:1">
+      <c r="A75" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="76" spans="1:1">
+      <c r="A76" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="77" spans="1:1">
+      <c r="A77" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="78" spans="1:1">
+      <c r="A78" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="79" spans="1:1">
+      <c r="A79" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="81" spans="1:1">
+      <c r="A81" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="83" spans="1:1">
+      <c r="A83" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="87" spans="1:1" ht="23.25">
+      <c r="A87" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="89" spans="1:1">
+      <c r="A89" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="91" spans="1:1">
+      <c r="A91" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="93" spans="1:1">
+      <c r="A93" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="94" spans="1:1">
+      <c r="A94" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="95" spans="1:1">
+      <c r="A95" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="96" spans="1:1">
+      <c r="A96" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="97" spans="1:1">
+      <c r="A97" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="99" spans="1:1">
+      <c r="A99" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="103" spans="1:1" ht="23.25">
+      <c r="A103" s="2" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="105" spans="1:1">
+      <c r="A105" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="107" spans="1:1">
+      <c r="A107" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="109" spans="1:1">
+      <c r="A109" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="110" spans="1:1">
+      <c r="A110" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="111" spans="1:1">
+      <c r="A111" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="112" spans="1:1">
+      <c r="A112" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="113" spans="1:1">
+      <c r="A113" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="114" spans="1:1">
+      <c r="A114" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="118" spans="1:1" ht="23.25">
+      <c r="A118" s="2" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="120" spans="1:1">
+      <c r="A120" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="122" spans="1:1">
+      <c r="A122" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="124" spans="1:1">
+      <c r="A124" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="125" spans="1:1">
+      <c r="A125" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="126" spans="1:1">
+      <c r="A126" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="127" spans="1:1">
+      <c r="A127" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="128" spans="1:1">
+      <c r="A128" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="129" spans="1:1">
+      <c r="A129" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="130" spans="1:1">
+      <c r="A130" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="132" spans="1:1">
+      <c r="A132" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="136" spans="1:1" ht="23.25">
+      <c r="A136" s="2" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="138" spans="1:1">
+      <c r="A138" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="140" spans="1:1">
+      <c r="A140" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="142" spans="1:1">
+      <c r="A142" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="143" spans="1:1">
+      <c r="A143" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="144" spans="1:1">
+      <c r="A144" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="145" spans="1:1">
+      <c r="A145" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="146" spans="1:1">
+      <c r="A146" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="148" spans="1:1">
+      <c r="A148" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="152" spans="1:1" ht="31.5">
+      <c r="A152" s="1" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="154" spans="1:1">
+      <c r="A154" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="156" spans="1:1">
+      <c r="A156" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="158" spans="1:1">
+      <c r="A158" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="160" spans="1:1">
+      <c r="A160" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="162" spans="1:1">
+      <c r="A162" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="164" spans="1:1">
+      <c r="A164" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="168" spans="1:1" ht="31.5">
+      <c r="A168" s="1" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="170" spans="1:1">
+      <c r="A170" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="172" spans="1:1">
+      <c r="A172" s="3" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="174" spans="1:1">
+      <c r="A174" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="176" spans="1:1">
+      <c r="A176" s="3" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="180" spans="1:1" ht="31.5">
+      <c r="A180" s="1" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="182" spans="1:1">
+      <c r="A182" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="184" spans="1:1">
+      <c r="A184" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="185" spans="1:1">
+      <c r="A185" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="24" spans="1:1" ht="17" x14ac:dyDescent="0.25">
-      <c r="A24" s="3" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="25" spans="1:1" ht="17" x14ac:dyDescent="0.25">
-      <c r="A25" s="3" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="26" spans="1:1" ht="17" x14ac:dyDescent="0.25">
-      <c r="A26" s="3" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="27" spans="1:1" ht="17" x14ac:dyDescent="0.25">
-      <c r="A27" s="3" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="28" spans="1:1" ht="17" x14ac:dyDescent="0.25">
-      <c r="A28" s="3" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="29" spans="1:1" ht="17" x14ac:dyDescent="0.25">
-      <c r="A29" s="3" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="30" spans="1:1" ht="17" x14ac:dyDescent="0.25">
-      <c r="A30" s="3" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="31" spans="1:1" ht="17" x14ac:dyDescent="0.25">
-      <c r="A31" s="3" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="32" spans="1:1" ht="17" x14ac:dyDescent="0.25">
-      <c r="A32" s="3" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="33" spans="1:1" ht="17" x14ac:dyDescent="0.25">
-      <c r="A33" s="3" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="34" spans="1:1" ht="17" x14ac:dyDescent="0.25">
-      <c r="A34" s="3" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="38" spans="1:1" ht="31" x14ac:dyDescent="0.35">
-      <c r="A38" s="1" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="40" spans="1:1" ht="24" x14ac:dyDescent="0.3">
-      <c r="A40" s="2" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A42" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A44" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A46" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A47" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A48" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A49" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A50" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A51" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A52" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A53" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A54" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A55" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A56" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="57" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A57" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="58" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A58" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="60" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A60" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="62" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A62" s="4" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="66" spans="1:1" ht="24" x14ac:dyDescent="0.3">
-      <c r="A66" s="2" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="68" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A68" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="70" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A70" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="72" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A72" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="74" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A74" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="75" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A75" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="76" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A76" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="77" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A77" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="78" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A78" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="79" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A79" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="81" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A81" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="83" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A83" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="87" spans="1:1" ht="24" x14ac:dyDescent="0.3">
-      <c r="A87" s="2" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="89" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A89" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="91" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A91" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="93" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A93" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="94" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A94" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="95" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A95" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="96" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A96" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="97" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A97" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="99" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A99" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="103" spans="1:1" ht="24" x14ac:dyDescent="0.3">
-      <c r="A103" s="2" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="105" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A105" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="107" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A107" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="109" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A109" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="110" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A110" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="111" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A111" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="112" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A112" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="113" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A113" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="114" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A114" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="118" spans="1:1" ht="24" x14ac:dyDescent="0.3">
-      <c r="A118" s="2" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="120" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A120" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="122" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A122" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="124" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A124" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="125" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A125" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="126" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A126" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="127" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A127" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="128" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A128" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="129" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A129" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="130" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A130" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="132" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A132" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="136" spans="1:1" ht="24" x14ac:dyDescent="0.3">
-      <c r="A136" s="2" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="138" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A138" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="140" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A140" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="142" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A142" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="143" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A143" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="144" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A144" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="145" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A145" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="146" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A146" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="148" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A148" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="152" spans="1:1" ht="31" x14ac:dyDescent="0.35">
-      <c r="A152" s="1" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="154" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A154" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="156" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A156" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="158" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A158" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="160" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A160" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="162" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A162" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="164" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A164" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="168" spans="1:1" ht="31" x14ac:dyDescent="0.35">
-      <c r="A168" s="1" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="170" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A170" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="172" spans="1:1" ht="17" x14ac:dyDescent="0.25">
-      <c r="A172" s="3" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="174" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A174" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="176" spans="1:1" ht="17" x14ac:dyDescent="0.25">
-      <c r="A176" s="3" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="180" spans="1:1" ht="31" x14ac:dyDescent="0.35">
-      <c r="A180" s="1" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="182" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A182" t="s">
+    <row r="186" spans="1:1">
+      <c r="A186" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="184" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A184" t="s">
+    <row r="187" spans="1:1">
+      <c r="A187" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="185" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A185" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="186" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A186" t="s">
+    <row r="188" spans="1:1">
+      <c r="A188" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="187" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A187" t="s">
+    <row r="190" spans="1:1">
+      <c r="A190" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="188" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A188" t="s">
+    <row r="194" spans="1:1" ht="31.5">
+      <c r="A194" s="1" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="190" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A190" t="s">
+    <row r="196" spans="1:1">
+      <c r="A196" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="194" spans="1:1" ht="31" x14ac:dyDescent="0.35">
-      <c r="A194" s="1" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="196" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A196" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="198" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="198" spans="1:1">
       <c r="A198" s="4">
         <v>4</v>
       </c>
     </row>
-    <row r="200" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="200" spans="1:1">
       <c r="A200" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="202" spans="1:1">
+      <c r="A202" s="4" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="204" spans="1:1">
+      <c r="A204" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="202" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A202" s="4" t="s">
+    <row r="206" spans="1:1">
+      <c r="A206" s="4" t="s">
         <v>146</v>
-      </c>
-    </row>
-    <row r="204" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A204" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="206" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A206" s="4" t="s">
-        <v>148</v>
       </c>
     </row>
   </sheetData>
@@ -3542,32 +3502,32 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{71908A3D-5F77-7940-A0CC-4753EB31826E}">
   <dimension ref="A1:V1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75"/>
   <cols>
-    <col min="1" max="1" width="7.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12.5" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="7" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="9.5" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="6.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="6.33203125" customWidth="1"/>
-    <col min="8" max="8" width="11.33203125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="7.6640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="13.6640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.6640625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="18.33203125" customWidth="1"/>
-    <col min="14" max="14" width="21.1640625" customWidth="1"/>
-    <col min="15" max="15" width="10.6640625" customWidth="1"/>
+    <col min="6" max="6" width="6.375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.375" customWidth="1"/>
+    <col min="8" max="8" width="11.375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="7.625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="18.375" customWidth="1"/>
+    <col min="14" max="14" width="21.125" customWidth="1"/>
+    <col min="15" max="15" width="10.625" customWidth="1"/>
     <col min="16" max="16" width="12" customWidth="1"/>
-    <col min="17" max="17" width="11.83203125" customWidth="1"/>
-    <col min="18" max="18" width="13.83203125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="13.1640625" customWidth="1"/>
+    <col min="17" max="17" width="11.875" customWidth="1"/>
+    <col min="18" max="18" width="13.875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="12.375" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="13.125" customWidth="1"/>
     <col min="21" max="22" width="10.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:22">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
@@ -3587,7 +3547,7 @@
         <v>5</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="H1" s="5" t="s">
         <v>6</v>
@@ -3605,31 +3565,31 @@
         <v>16</v>
       </c>
       <c r="M1" s="5" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="N1" s="5" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="O1" s="5" t="s">
         <v>17</v>
       </c>
       <c r="P1" s="5" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="Q1" s="5" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="R1" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="S1" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="T1" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="S1" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="T1" s="5" t="s">
+      <c r="U1" s="5" t="s">
         <v>28</v>
-      </c>
-      <c r="U1" s="5" t="s">
-        <v>29</v>
       </c>
       <c r="V1" s="5" t="s">
         <v>11</v>
@@ -3643,47 +3603,47 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{78E98199-A67A-9349-9480-7BF0BBC64AD0}">
   <dimension ref="A1:Q1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75"/>
   <cols>
-    <col min="1" max="1" width="16.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.6640625" customWidth="1"/>
-    <col min="3" max="3" width="14.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.33203125" customWidth="1"/>
-    <col min="5" max="5" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="8" width="12.6640625" customWidth="1"/>
-    <col min="9" max="9" width="16.6640625" customWidth="1"/>
-    <col min="11" max="11" width="14.83203125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="14.83203125" customWidth="1"/>
-    <col min="14" max="14" width="12.83203125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="11.83203125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="12.83203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.625" customWidth="1"/>
+    <col min="3" max="3" width="14.375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.375" customWidth="1"/>
+    <col min="5" max="5" width="12.625" bestFit="1" customWidth="1"/>
+    <col min="6" max="8" width="12.625" customWidth="1"/>
+    <col min="9" max="9" width="16.625" customWidth="1"/>
+    <col min="11" max="11" width="14.875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="14.875" customWidth="1"/>
+    <col min="14" max="14" width="12.875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="11.875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="12.875" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="13" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:17">
       <c r="A1" s="5" t="s">
         <v>12</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="C1" s="5" t="s">
         <v>20</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="I1" s="5" t="s">
         <v>18</v>
@@ -3692,25 +3652,25 @@
         <v>19</v>
       </c>
       <c r="K1" s="5" t="s">
+        <v>288</v>
+      </c>
+      <c r="L1" s="5" t="s">
         <v>290</v>
       </c>
-      <c r="L1" s="5" t="s">
-        <v>292</v>
-      </c>
       <c r="M1" s="5" t="s">
+        <v>289</v>
+      </c>
+      <c r="N1" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="O1" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="P1" s="5" t="s">
         <v>291</v>
       </c>
-      <c r="N1" s="5" t="s">
-        <v>149</v>
-      </c>
-      <c r="O1" s="5" t="s">
-        <v>150</v>
-      </c>
-      <c r="P1" s="5" t="s">
-        <v>293</v>
-      </c>
       <c r="Q1" s="5" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
     </row>
   </sheetData>
@@ -3721,27 +3681,27 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7BEE41B9-5039-F448-A0EF-8770476CF667}">
   <dimension ref="A1:P1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75"/>
   <cols>
-    <col min="1" max="1" width="15.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.33203125" customWidth="1"/>
-    <col min="3" max="3" width="14.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.1640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.375" customWidth="1"/>
+    <col min="3" max="3" width="14.375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.375" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="14" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.6640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="6.83203125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="9.1640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="6.875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9.125" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="6" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="9.5" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="17.1640625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="10.1640625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="17.125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="10.125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:16">
       <c r="A1" s="5" t="s">
         <v>12</v>
       </c>
@@ -3755,16 +3715,16 @@
         <v>16</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="F1" s="5" t="s">
+        <v>316</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>317</v>
+      </c>
+      <c r="H1" s="5" t="s">
         <v>318</v>
-      </c>
-      <c r="G1" s="5" t="s">
-        <v>319</v>
-      </c>
-      <c r="H1" s="5" t="s">
-        <v>320</v>
       </c>
       <c r="I1" s="5" t="s">
         <v>19</v>
@@ -3782,10 +3742,10 @@
         <v>5</v>
       </c>
       <c r="N1" s="5" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="O1" s="5" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="P1" s="5" t="s">
         <v>17</v>
@@ -3800,31 +3760,31 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6B5A506-ED07-C540-BAA9-C3B85D3BE076}">
   <dimension ref="A1:X1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75"/>
   <cols>
-    <col min="1" max="1" width="15.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="7.5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.1640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.375" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="14" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="14" customWidth="1"/>
-    <col min="9" max="9" width="16.83203125" bestFit="1" customWidth="1"/>
-    <col min="10" max="11" width="16.83203125" customWidth="1"/>
+    <col min="9" max="9" width="16.875" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="16.875" customWidth="1"/>
     <col min="12" max="12" width="14" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="14" customWidth="1"/>
     <col min="14" max="14" width="18" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="15.1640625" bestFit="1" customWidth="1"/>
-    <col min="16" max="17" width="15.1640625" customWidth="1"/>
-    <col min="18" max="18" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="22.83203125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="5.6640625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="15.125" bestFit="1" customWidth="1"/>
+    <col min="16" max="17" width="15.125" customWidth="1"/>
+    <col min="18" max="18" width="12.375" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="22.875" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="5.625" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="10" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="14.375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:24">
       <c r="A1" s="5" t="s">
         <v>12</v>
       </c>
@@ -3838,61 +3798,61 @@
         <v>16</v>
       </c>
       <c r="E1" s="5" t="s">
+        <v>320</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>316</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>317</v>
+      </c>
+      <c r="H1" s="9" t="s">
+        <v>352</v>
+      </c>
+      <c r="I1" s="5" t="s">
+        <v>321</v>
+      </c>
+      <c r="J1" s="9" t="s">
+        <v>355</v>
+      </c>
+      <c r="K1" s="5" t="s">
+        <v>356</v>
+      </c>
+      <c r="L1" s="5" t="s">
+        <v>282</v>
+      </c>
+      <c r="M1" s="5" t="s">
         <v>322</v>
       </c>
-      <c r="F1" s="5" t="s">
-        <v>318</v>
-      </c>
-      <c r="G1" s="5" t="s">
-        <v>319</v>
-      </c>
-      <c r="H1" s="9" t="s">
-        <v>357</v>
-      </c>
-      <c r="I1" s="5" t="s">
-        <v>323</v>
-      </c>
-      <c r="J1" s="9" t="s">
-        <v>360</v>
-      </c>
-      <c r="K1" s="5" t="s">
-        <v>361</v>
-      </c>
-      <c r="L1" s="5" t="s">
-        <v>284</v>
-      </c>
-      <c r="M1" s="5" t="s">
-        <v>324</v>
-      </c>
       <c r="N1" s="5" t="s">
-        <v>356</v>
+        <v>351</v>
       </c>
       <c r="O1" s="5" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="P1" s="5" t="s">
-        <v>359</v>
+        <v>354</v>
       </c>
       <c r="Q1" s="9" t="s">
-        <v>358</v>
+        <v>353</v>
       </c>
       <c r="R1" s="5" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="S1" s="5" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="T1" s="5" t="s">
-        <v>341</v>
+        <v>336</v>
       </c>
       <c r="U1" s="5" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="V1" s="5" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="W1" s="5" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="X1" s="5"/>
     </row>
@@ -3905,7 +3865,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C9C37EAA-1416-4F4A-AF23-179144E9C194}">
   <dimension ref="A1:L1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="20" style="7" customWidth="1"/>
     <col min="2" max="6" width="18" style="7" customWidth="1"/>
@@ -3913,11 +3873,11 @@
     <col min="8" max="8" width="20" style="7" customWidth="1"/>
     <col min="9" max="9" width="19" style="7" customWidth="1"/>
     <col min="10" max="11" width="20" style="7" customWidth="1"/>
-    <col min="12" max="12" width="8.1640625" style="7" bestFit="1" customWidth="1"/>
-    <col min="13" max="16384" width="8.83203125" style="7"/>
+    <col min="12" max="12" width="8.125" style="7" bestFit="1" customWidth="1"/>
+    <col min="13" max="16384" width="8.875" style="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:12">
       <c r="A1" s="6" t="s">
         <v>12</v>
       </c>
@@ -3925,34 +3885,34 @@
         <v>13</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="D1" s="6" t="s">
+        <v>292</v>
+      </c>
+      <c r="E1" s="6" t="s">
         <v>294</v>
       </c>
-      <c r="E1" s="6" t="s">
-        <v>296</v>
-      </c>
       <c r="F1" s="6" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>363</v>
+        <v>358</v>
       </c>
       <c r="H1" s="6" t="s">
-        <v>362</v>
+        <v>357</v>
       </c>
       <c r="I1" s="6" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="J1" s="6" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="K1" s="6" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="L1" s="6" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -3964,16 +3924,16 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA73BFB8-99EA-FA4A-B1AD-DB3F1F0EC303}">
   <dimension ref="A1:N1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="20" style="7" customWidth="1"/>
     <col min="2" max="11" width="18" style="7" customWidth="1"/>
-    <col min="12" max="12" width="9.1640625" style="7" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="9.1640625" style="7" customWidth="1"/>
-    <col min="14" max="16384" width="8.83203125" style="7"/>
+    <col min="12" max="12" width="9.125" style="7" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="9.125" style="7" customWidth="1"/>
+    <col min="14" max="16384" width="8.875" style="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:14">
       <c r="A1" s="6" t="s">
         <v>12</v>
       </c>
@@ -3981,40 +3941,40 @@
         <v>13</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="E1" s="6" t="s">
+        <v>322</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>302</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="H1" s="6" t="s">
+        <v>282</v>
+      </c>
+      <c r="I1" s="6" t="s">
+        <v>239</v>
+      </c>
+      <c r="J1" s="6" t="s">
+        <v>281</v>
+      </c>
+      <c r="K1" s="6" t="s">
+        <v>296</v>
+      </c>
+      <c r="L1" s="6" t="s">
+        <v>280</v>
+      </c>
+      <c r="M1" s="6" t="s">
+        <v>323</v>
+      </c>
+      <c r="N1" s="6" t="s">
         <v>324</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>304</v>
-      </c>
-      <c r="G1" s="5" t="s">
-        <v>152</v>
-      </c>
-      <c r="H1" s="6" t="s">
-        <v>284</v>
-      </c>
-      <c r="I1" s="6" t="s">
-        <v>241</v>
-      </c>
-      <c r="J1" s="6" t="s">
-        <v>283</v>
-      </c>
-      <c r="K1" s="6" t="s">
-        <v>298</v>
-      </c>
-      <c r="L1" s="6" t="s">
-        <v>282</v>
-      </c>
-      <c r="M1" s="6" t="s">
-        <v>325</v>
-      </c>
-      <c r="N1" s="6" t="s">
-        <v>326</v>
       </c>
     </row>
   </sheetData>
@@ -4026,18 +3986,18 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{268F324C-9C8C-3D42-A9E2-08CDCD4510B5}">
   <dimension ref="A1:I1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75"/>
   <cols>
-    <col min="1" max="1" width="15.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.83203125" customWidth="1"/>
-    <col min="3" max="3" width="17.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.6640625" customWidth="1"/>
+    <col min="1" max="1" width="15.375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.875" customWidth="1"/>
+    <col min="3" max="3" width="17.375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.625" customWidth="1"/>
     <col min="6" max="6" width="15" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.83203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9">
       <c r="A1" s="6" t="s">
         <v>12</v>
       </c>
@@ -4045,25 +4005,25 @@
         <v>13</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="H1" s="6" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="I1" s="6" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
     </row>
   </sheetData>
@@ -4075,17 +4035,17 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{071B2430-B111-D04E-8A80-272CE176271D}">
   <dimension ref="A1:M1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75"/>
   <cols>
     <col min="3" max="3" width="14.5" customWidth="1"/>
-    <col min="4" max="5" width="18.1640625" customWidth="1"/>
+    <col min="4" max="5" width="18.125" customWidth="1"/>
     <col min="6" max="6" width="12.5" customWidth="1"/>
-    <col min="7" max="7" width="16.33203125" customWidth="1"/>
-    <col min="8" max="8" width="16.83203125" customWidth="1"/>
-    <col min="11" max="11" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.375" customWidth="1"/>
+    <col min="8" max="8" width="16.875" customWidth="1"/>
+    <col min="11" max="11" width="8.625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:13">
       <c r="A1" s="6" t="s">
         <v>12</v>
       </c>
@@ -4093,37 +4053,37 @@
         <v>13</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>343</v>
+        <v>338</v>
       </c>
       <c r="I1" s="5" t="s">
-        <v>344</v>
+        <v>339</v>
       </c>
       <c r="J1" s="5" t="s">
-        <v>345</v>
+        <v>340</v>
       </c>
       <c r="K1" s="5" t="s">
-        <v>346</v>
+        <v>341</v>
       </c>
       <c r="L1" s="5" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="M1" s="5" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
     </row>
   </sheetData>

</xml_diff>